<commit_message>
yolo fir ve terhmal bitti
</commit_message>
<xml_diff>
--- a/runs/yolo_fir_v5s_28.05.2026/training_metrics.xlsx
+++ b/runs/yolo_fir_v5s_28.05.2026/training_metrics.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y7"/>
+  <dimension ref="A1:Y47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -982,6 +982,2360 @@
       <c r="X7" s="5" t="n"/>
       <c r="Y7" s="5" t="n"/>
     </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>0.004715</v>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>1.3989</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1.4098</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>0.6503</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>0.7924</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>0.8913</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>0.8027</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>0.7504</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>0.7756999999999999</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>0.7877999999999999</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>0.5102</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>0.9046</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>0.4749</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0.9165</v>
+      </c>
+      <c r="Q8" s="4" t="n"/>
+      <c r="R8" s="4" t="n"/>
+      <c r="S8" s="4" t="n"/>
+      <c r="T8" s="4" t="n"/>
+      <c r="U8" s="4" t="n"/>
+      <c r="V8" s="4" t="n"/>
+      <c r="W8" s="4" t="n"/>
+      <c r="X8" s="4" t="n"/>
+      <c r="Y8" s="4" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>0.0046675</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>1.4069</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>1.3706</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>0.6961000000000001</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0.7737000000000001</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0.8651</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>0.8857</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>0.7232</v>
+      </c>
+      <c r="J9" s="5" t="n">
+        <v>0.7704</v>
+      </c>
+      <c r="K9" s="5" t="n">
+        <v>0.7461</v>
+      </c>
+      <c r="L9" s="5" t="n">
+        <v>0.7509</v>
+      </c>
+      <c r="M9" s="5" t="n">
+        <v>0.4962</v>
+      </c>
+      <c r="N9" s="5" t="n">
+        <v>0.9127999999999999</v>
+      </c>
+      <c r="O9" s="5" t="n">
+        <v>0.4936</v>
+      </c>
+      <c r="P9" s="5" t="n">
+        <v>0.8677</v>
+      </c>
+      <c r="Q9" s="5" t="n"/>
+      <c r="R9" s="5" t="n"/>
+      <c r="S9" s="5" t="n"/>
+      <c r="T9" s="5" t="n"/>
+      <c r="U9" s="5" t="n"/>
+      <c r="V9" s="5" t="n"/>
+      <c r="W9" s="5" t="n"/>
+      <c r="X9" s="5" t="n"/>
+      <c r="Y9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>0.00462</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>1.4347</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1.3514</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>0.7201</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0.7567</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>0.9550999999999999</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>0.7204</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>0.767</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0.743</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>0.748</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>0.9183</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>0.4976</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0.8848</v>
+      </c>
+      <c r="Q10" s="4" t="n"/>
+      <c r="R10" s="4" t="n"/>
+      <c r="S10" s="4" t="n"/>
+      <c r="T10" s="4" t="n"/>
+      <c r="U10" s="4" t="n"/>
+      <c r="V10" s="4" t="n"/>
+      <c r="W10" s="4" t="n"/>
+      <c r="X10" s="4" t="n"/>
+      <c r="Y10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>0.0045725</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>1.4217</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>1.3445</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>0.7226</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0.7482</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0.8905999999999999</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>0.8819</v>
+      </c>
+      <c r="I11" s="5" t="n">
+        <v>0.7425</v>
+      </c>
+      <c r="J11" s="5" t="n">
+        <v>0.8175</v>
+      </c>
+      <c r="K11" s="5" t="n">
+        <v>0.7782</v>
+      </c>
+      <c r="L11" s="5" t="n">
+        <v>0.7863</v>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>0.5332</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>0.923</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>0.5076000000000001</v>
+      </c>
+      <c r="P11" s="5" t="n">
+        <v>0.8767</v>
+      </c>
+      <c r="Q11" s="5" t="n"/>
+      <c r="R11" s="5" t="n"/>
+      <c r="S11" s="5" t="n"/>
+      <c r="T11" s="5" t="n"/>
+      <c r="U11" s="5" t="n"/>
+      <c r="V11" s="5" t="n"/>
+      <c r="W11" s="5" t="n"/>
+      <c r="X11" s="5" t="n"/>
+      <c r="Y11" s="5" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>0.004525</v>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>1.1902</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>1.3148</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>0.5747</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>0.7357</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>0.856</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>0.876</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>0.7498</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>0.7261</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0.7377</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>0.751</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>0.5065</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>0.924</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>0.518</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0.9086</v>
+      </c>
+      <c r="Q12" s="4" t="n"/>
+      <c r="R12" s="4" t="n"/>
+      <c r="S12" s="4" t="n"/>
+      <c r="T12" s="4" t="n"/>
+      <c r="U12" s="4" t="n"/>
+      <c r="V12" s="4" t="n"/>
+      <c r="W12" s="4" t="n"/>
+      <c r="X12" s="4" t="n"/>
+      <c r="Y12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>0.0044775</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>1.502</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>1.3078</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>0.7104</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0.7216</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0.917</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>0.8745000000000001</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>0.6904</v>
+      </c>
+      <c r="J13" s="5" t="n">
+        <v>0.8011</v>
+      </c>
+      <c r="K13" s="5" t="n">
+        <v>0.7416</v>
+      </c>
+      <c r="L13" s="5" t="n">
+        <v>0.7753</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>0.5339</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>0.9266</v>
+      </c>
+      <c r="O13" s="5" t="n">
+        <v>0.5178</v>
+      </c>
+      <c r="P13" s="5" t="n">
+        <v>0.8443000000000001</v>
+      </c>
+      <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="5" t="n"/>
+      <c r="S13" s="5" t="n"/>
+      <c r="T13" s="5" t="n"/>
+      <c r="U13" s="5" t="n"/>
+      <c r="V13" s="5" t="n"/>
+      <c r="W13" s="5" t="n"/>
+      <c r="X13" s="5" t="n"/>
+      <c r="Y13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>0.00443</v>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>1.1966</v>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1.2988</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>0.7234</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>0.9179</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>0.8729</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>0.7914</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>0.7594</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>0.7751</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>0.8093</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>0.5587</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>0.9294</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>0.5177</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0.9176</v>
+      </c>
+      <c r="Q14" s="4" t="n"/>
+      <c r="R14" s="4" t="n"/>
+      <c r="S14" s="4" t="n"/>
+      <c r="T14" s="4" t="n"/>
+      <c r="U14" s="4" t="n"/>
+      <c r="V14" s="4" t="n"/>
+      <c r="W14" s="4" t="n"/>
+      <c r="X14" s="4" t="n"/>
+      <c r="Y14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>0.0043825</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>1.4043</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>1.2859</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>0.6074000000000001</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0.7122000000000001</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0.8079</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>0.8693</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>0.7737000000000001</v>
+      </c>
+      <c r="J15" s="5" t="n">
+        <v>0.8090000000000001</v>
+      </c>
+      <c r="K15" s="5" t="n">
+        <v>0.7909</v>
+      </c>
+      <c r="L15" s="5" t="n">
+        <v>0.8052</v>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>0.5581</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>0.9321</v>
+      </c>
+      <c r="O15" s="5" t="n">
+        <v>0.5256999999999999</v>
+      </c>
+      <c r="P15" s="5" t="n">
+        <v>0.9034</v>
+      </c>
+      <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="5" t="n"/>
+      <c r="S15" s="5" t="n"/>
+      <c r="T15" s="5" t="n"/>
+      <c r="U15" s="5" t="n"/>
+      <c r="V15" s="5" t="n"/>
+      <c r="W15" s="5" t="n"/>
+      <c r="X15" s="5" t="n"/>
+      <c r="Y15" s="5" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>0.004335</v>
+      </c>
+      <c r="C16" s="4" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>1.2765</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>0.5618</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>0.7036</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>0.8548</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>0.8689</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>0.8258</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>0.8003</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>0.8129</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>0.8201000000000001</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>0.5721000000000001</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>0.9376</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>0.5318000000000001</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0.9292</v>
+      </c>
+      <c r="Q16" s="4" t="n"/>
+      <c r="R16" s="4" t="n"/>
+      <c r="S16" s="4" t="n"/>
+      <c r="T16" s="4" t="n"/>
+      <c r="U16" s="4" t="n"/>
+      <c r="V16" s="4" t="n"/>
+      <c r="W16" s="4" t="n"/>
+      <c r="X16" s="4" t="n"/>
+      <c r="Y16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>0.0042875</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>1.2572</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>1.2669</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>0.5823</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0.6962</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0.8439</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>0.7573</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>0.8277</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>0.7909</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>0.7995</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>0.5570000000000001</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>0.9381</v>
+      </c>
+      <c r="O17" s="5" t="n">
+        <v>0.5332</v>
+      </c>
+      <c r="P17" s="5" t="n">
+        <v>0.887</v>
+      </c>
+      <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="5" t="n"/>
+      <c r="S17" s="5" t="n"/>
+      <c r="T17" s="5" t="n"/>
+      <c r="U17" s="5" t="n"/>
+      <c r="V17" s="5" t="n"/>
+      <c r="W17" s="5" t="n"/>
+      <c r="X17" s="5" t="n"/>
+      <c r="Y17" s="5" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>0.00424</v>
+      </c>
+      <c r="C18" s="4" t="n">
+        <v>1.1589</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>1.2602</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>0.5921999999999999</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>0.6904</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0.8285</v>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>0.8657</v>
+      </c>
+      <c r="I18" s="4" t="n">
+        <v>0.7547</v>
+      </c>
+      <c r="J18" s="4" t="n">
+        <v>0.8379</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>0.7942</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>0.7994</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>0.5622</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>0.9402</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>0.5365</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>0.8915</v>
+      </c>
+      <c r="Q18" s="4" t="n"/>
+      <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="n"/>
+      <c r="T18" s="4" t="n"/>
+      <c r="U18" s="4" t="n"/>
+      <c r="V18" s="4" t="n"/>
+      <c r="W18" s="4" t="n"/>
+      <c r="X18" s="4" t="n"/>
+      <c r="Y18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>0.0041925</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>1.414</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>1.2557</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0.6685</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0.6870000000000001</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0.8194</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0.865</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>0.8242</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>0.7798</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>0.7968</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>0.5602</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>0.9412</v>
+      </c>
+      <c r="O19" s="5" t="n">
+        <v>0.5386</v>
+      </c>
+      <c r="P19" s="5" t="n">
+        <v>0.8852</v>
+      </c>
+      <c r="Q19" s="5" t="n"/>
+      <c r="R19" s="5" t="n"/>
+      <c r="S19" s="5" t="n"/>
+      <c r="T19" s="5" t="n"/>
+      <c r="U19" s="5" t="n"/>
+      <c r="V19" s="5" t="n"/>
+      <c r="W19" s="5" t="n"/>
+      <c r="X19" s="5" t="n"/>
+      <c r="Y19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="n">
+        <v>0.004145</v>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>1.1819</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>1.2534</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>0.5457</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>0.6857</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>0.8542</v>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>0.8643</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0.7561</v>
+      </c>
+      <c r="J20" s="4" t="n">
+        <v>0.8021</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>0.7784</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>0.7984</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>0.5595</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>0.9409</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>0.5401</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>0.9164</v>
+      </c>
+      <c r="Q20" s="4" t="n"/>
+      <c r="R20" s="4" t="n"/>
+      <c r="S20" s="4" t="n"/>
+      <c r="T20" s="4" t="n"/>
+      <c r="U20" s="4" t="n"/>
+      <c r="V20" s="4" t="n"/>
+      <c r="W20" s="4" t="n"/>
+      <c r="X20" s="4" t="n"/>
+      <c r="Y20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>0.0040975</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>0.9641</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>1.2521</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>0.4955</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0.6831</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>0.8502</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>0.8636</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>0.7294</v>
+      </c>
+      <c r="J21" s="5" t="n">
+        <v>0.8152</v>
+      </c>
+      <c r="K21" s="5" t="n">
+        <v>0.7699</v>
+      </c>
+      <c r="L21" s="5" t="n">
+        <v>0.7965</v>
+      </c>
+      <c r="M21" s="5" t="n">
+        <v>0.5595</v>
+      </c>
+      <c r="N21" s="5" t="n">
+        <v>0.9421</v>
+      </c>
+      <c r="O21" s="5" t="n">
+        <v>0.5411</v>
+      </c>
+      <c r="P21" s="5" t="n">
+        <v>0.8883</v>
+      </c>
+      <c r="Q21" s="5" t="n"/>
+      <c r="R21" s="5" t="n"/>
+      <c r="S21" s="5" t="n"/>
+      <c r="T21" s="5" t="n"/>
+      <c r="U21" s="5" t="n"/>
+      <c r="V21" s="5" t="n"/>
+      <c r="W21" s="5" t="n"/>
+      <c r="X21" s="5" t="n"/>
+      <c r="Y21" s="5" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4" t="n">
+        <v>0.00405</v>
+      </c>
+      <c r="C22" s="4" t="n">
+        <v>1.3529</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>1.2489</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>0.7181</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>0.6795</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>0.8848</v>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>0.863</v>
+      </c>
+      <c r="I22" s="4" t="n">
+        <v>0.7422</v>
+      </c>
+      <c r="J22" s="4" t="n">
+        <v>0.8013</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>0.7706</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>0.8025</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>0.5674</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>0.9423</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>0.5417999999999999</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>0.8957000000000001</v>
+      </c>
+      <c r="Q22" s="4" t="n"/>
+      <c r="R22" s="4" t="n"/>
+      <c r="S22" s="4" t="n"/>
+      <c r="T22" s="4" t="n"/>
+      <c r="U22" s="4" t="n"/>
+      <c r="V22" s="4" t="n"/>
+      <c r="W22" s="4" t="n"/>
+      <c r="X22" s="4" t="n"/>
+      <c r="Y22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>0.0040025</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>1.1195</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>1.2476</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>0.5433</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0.6774</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0.9028</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>0.8626</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>0.7645999999999999</v>
+      </c>
+      <c r="J23" s="5" t="n">
+        <v>0.7935</v>
+      </c>
+      <c r="K23" s="5" t="n">
+        <v>0.7788</v>
+      </c>
+      <c r="L23" s="5" t="n">
+        <v>0.8018999999999999</v>
+      </c>
+      <c r="M23" s="5" t="n">
+        <v>0.5658</v>
+      </c>
+      <c r="N23" s="5" t="n">
+        <v>0.9428</v>
+      </c>
+      <c r="O23" s="5" t="n">
+        <v>0.5433</v>
+      </c>
+      <c r="P23" s="5" t="n">
+        <v>0.9145</v>
+      </c>
+      <c r="Q23" s="5" t="n"/>
+      <c r="R23" s="5" t="n"/>
+      <c r="S23" s="5" t="n"/>
+      <c r="T23" s="5" t="n"/>
+      <c r="U23" s="5" t="n"/>
+      <c r="V23" s="5" t="n"/>
+      <c r="W23" s="5" t="n"/>
+      <c r="X23" s="5" t="n"/>
+      <c r="Y23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="4" t="n">
+        <v>0.003955</v>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>0.9732</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>1.2442</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>0.4416</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>0.676</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0.8177</v>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>0.8619</v>
+      </c>
+      <c r="I24" s="4" t="n">
+        <v>0.7662</v>
+      </c>
+      <c r="J24" s="4" t="n">
+        <v>0.7956</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>0.7806</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>0.8043</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>0.5672</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>0.9431</v>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>0.5444</v>
+      </c>
+      <c r="P24" s="4" t="n">
+        <v>0.9132</v>
+      </c>
+      <c r="Q24" s="4" t="n"/>
+      <c r="R24" s="4" t="n"/>
+      <c r="S24" s="4" t="n"/>
+      <c r="T24" s="4" t="n"/>
+      <c r="U24" s="4" t="n"/>
+      <c r="V24" s="4" t="n"/>
+      <c r="W24" s="4" t="n"/>
+      <c r="X24" s="4" t="n"/>
+      <c r="Y24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>0.0039075</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>1.2938</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>1.2427</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>0.6081</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0.6744</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0.8381999999999999</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>0.8616</v>
+      </c>
+      <c r="I25" s="5" t="n">
+        <v>0.7121</v>
+      </c>
+      <c r="J25" s="5" t="n">
+        <v>0.8268</v>
+      </c>
+      <c r="K25" s="5" t="n">
+        <v>0.7652</v>
+      </c>
+      <c r="L25" s="5" t="n">
+        <v>0.8027</v>
+      </c>
+      <c r="M25" s="5" t="n">
+        <v>0.5664</v>
+      </c>
+      <c r="N25" s="5" t="n">
+        <v>0.9429999999999999</v>
+      </c>
+      <c r="O25" s="5" t="n">
+        <v>0.5449000000000001</v>
+      </c>
+      <c r="P25" s="5" t="n">
+        <v>0.8594000000000001</v>
+      </c>
+      <c r="Q25" s="5" t="n"/>
+      <c r="R25" s="5" t="n"/>
+      <c r="S25" s="5" t="n"/>
+      <c r="T25" s="5" t="n"/>
+      <c r="U25" s="5" t="n"/>
+      <c r="V25" s="5" t="n"/>
+      <c r="W25" s="5" t="n"/>
+      <c r="X25" s="5" t="n"/>
+      <c r="Y25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="4" t="n">
+        <v>0.00386</v>
+      </c>
+      <c r="C26" s="4" t="n">
+        <v>1.1066</v>
+      </c>
+      <c r="D26" s="4" t="n">
+        <v>1.2403</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>0.5642</v>
+      </c>
+      <c r="F26" s="4" t="n">
+        <v>0.6724</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>0.8358</v>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>0.8613</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>0.7846</v>
+      </c>
+      <c r="J26" s="4" t="n">
+        <v>0.7554</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>0.7697000000000001</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>0.7991</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>0.5634</v>
+      </c>
+      <c r="N26" s="4" t="n">
+        <v>0.944</v>
+      </c>
+      <c r="O26" s="4" t="n">
+        <v>0.5459000000000001</v>
+      </c>
+      <c r="P26" s="4" t="n">
+        <v>0.9409</v>
+      </c>
+      <c r="Q26" s="4" t="n"/>
+      <c r="R26" s="4" t="n"/>
+      <c r="S26" s="4" t="n"/>
+      <c r="T26" s="4" t="n"/>
+      <c r="U26" s="4" t="n"/>
+      <c r="V26" s="4" t="n"/>
+      <c r="W26" s="4" t="n"/>
+      <c r="X26" s="4" t="n"/>
+      <c r="Y26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>0.0038125</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>1.1862</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>1.2374</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>0.6203</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0.6716</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>0.9651</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>0.8608</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>0.7572</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>0.7654</v>
+      </c>
+      <c r="K27" s="5" t="n">
+        <v>0.7613</v>
+      </c>
+      <c r="L27" s="5" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="M27" s="5" t="n">
+        <v>0.5617</v>
+      </c>
+      <c r="N27" s="5" t="n">
+        <v>0.9439</v>
+      </c>
+      <c r="O27" s="5" t="n">
+        <v>0.5471</v>
+      </c>
+      <c r="P27" s="5" t="n">
+        <v>0.9191</v>
+      </c>
+      <c r="Q27" s="5" t="n"/>
+      <c r="R27" s="5" t="n"/>
+      <c r="S27" s="5" t="n"/>
+      <c r="T27" s="5" t="n"/>
+      <c r="U27" s="5" t="n"/>
+      <c r="V27" s="5" t="n"/>
+      <c r="W27" s="5" t="n"/>
+      <c r="X27" s="5" t="n"/>
+      <c r="Y27" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="4" t="n">
+        <v>0.003765</v>
+      </c>
+      <c r="C28" s="4" t="n">
+        <v>1.1985</v>
+      </c>
+      <c r="D28" s="4" t="n">
+        <v>1.2352</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>0.5979</v>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>0.6699000000000001</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0.8319</v>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>0.8606</v>
+      </c>
+      <c r="I28" s="4" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="J28" s="4" t="n">
+        <v>0.7651</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>0.7675</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>0.7943</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>0.5615</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>0.9445</v>
+      </c>
+      <c r="O28" s="4" t="n">
+        <v>0.5482</v>
+      </c>
+      <c r="P28" s="4" t="n">
+        <v>0.9232</v>
+      </c>
+      <c r="Q28" s="4" t="n"/>
+      <c r="R28" s="4" t="n"/>
+      <c r="S28" s="4" t="n"/>
+      <c r="T28" s="4" t="n"/>
+      <c r="U28" s="4" t="n"/>
+      <c r="V28" s="4" t="n"/>
+      <c r="W28" s="4" t="n"/>
+      <c r="X28" s="4" t="n"/>
+      <c r="Y28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>0.0037175</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>0.9897</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>1.2332</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>0.5138</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0.669</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>0.8316</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>0.8602</v>
+      </c>
+      <c r="I29" s="5" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="J29" s="5" t="n">
+        <v>0.8025</v>
+      </c>
+      <c r="K29" s="5" t="n">
+        <v>0.7602</v>
+      </c>
+      <c r="L29" s="5" t="n">
+        <v>0.7926</v>
+      </c>
+      <c r="M29" s="5" t="n">
+        <v>0.5608</v>
+      </c>
+      <c r="N29" s="5" t="n">
+        <v>0.9448</v>
+      </c>
+      <c r="O29" s="5" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="P29" s="5" t="n">
+        <v>0.8749</v>
+      </c>
+      <c r="Q29" s="5" t="n"/>
+      <c r="R29" s="5" t="n"/>
+      <c r="S29" s="5" t="n"/>
+      <c r="T29" s="5" t="n"/>
+      <c r="U29" s="5" t="n"/>
+      <c r="V29" s="5" t="n"/>
+      <c r="W29" s="5" t="n"/>
+      <c r="X29" s="5" t="n"/>
+      <c r="Y29" s="5" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="4" t="n">
+        <v>0.00367</v>
+      </c>
+      <c r="C30" s="4" t="n">
+        <v>0.9969</v>
+      </c>
+      <c r="D30" s="4" t="n">
+        <v>1.2328</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>0.5171</v>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>0.668</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>0.8288</v>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>0.8602</v>
+      </c>
+      <c r="I30" s="4" t="n">
+        <v>0.7907</v>
+      </c>
+      <c r="J30" s="4" t="n">
+        <v>0.7514</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>0.7706</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>0.7925</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>0.5607</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>0.9452</v>
+      </c>
+      <c r="O30" s="4" t="n">
+        <v>0.5506</v>
+      </c>
+      <c r="P30" s="4" t="n">
+        <v>0.9414</v>
+      </c>
+      <c r="Q30" s="4" t="n"/>
+      <c r="R30" s="4" t="n"/>
+      <c r="S30" s="4" t="n"/>
+      <c r="T30" s="4" t="n"/>
+      <c r="U30" s="4" t="n"/>
+      <c r="V30" s="4" t="n"/>
+      <c r="W30" s="4" t="n"/>
+      <c r="X30" s="4" t="n"/>
+      <c r="Y30" s="4" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>0.0036225</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>1.0901</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>1.2316</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>0.8315</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>0.7735</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>0.7587</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>0.7921</v>
+      </c>
+      <c r="M31" s="5" t="n">
+        <v>0.5599</v>
+      </c>
+      <c r="N31" s="5" t="n">
+        <v>0.9461000000000001</v>
+      </c>
+      <c r="O31" s="5" t="n">
+        <v>0.5508999999999999</v>
+      </c>
+      <c r="P31" s="5" t="n">
+        <v>0.9361</v>
+      </c>
+      <c r="Q31" s="5" t="n"/>
+      <c r="R31" s="5" t="n"/>
+      <c r="S31" s="5" t="n"/>
+      <c r="T31" s="5" t="n"/>
+      <c r="U31" s="5" t="n"/>
+      <c r="V31" s="5" t="n"/>
+      <c r="W31" s="5" t="n"/>
+      <c r="X31" s="5" t="n"/>
+      <c r="Y31" s="5" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="4" t="n">
+        <v>0.003575</v>
+      </c>
+      <c r="C32" s="4" t="n">
+        <v>1.1748</v>
+      </c>
+      <c r="D32" s="4" t="n">
+        <v>1.2308</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>0.5665</v>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>0.6666</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0.8524</v>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>0.8598</v>
+      </c>
+      <c r="I32" s="4" t="n">
+        <v>0.7781</v>
+      </c>
+      <c r="J32" s="4" t="n">
+        <v>0.7551</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>0.7664</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>0.7921</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>0.5603</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>0.9463</v>
+      </c>
+      <c r="O32" s="4" t="n">
+        <v>0.551</v>
+      </c>
+      <c r="P32" s="4" t="n">
+        <v>0.9397</v>
+      </c>
+      <c r="Q32" s="4" t="n"/>
+      <c r="R32" s="4" t="n"/>
+      <c r="S32" s="4" t="n"/>
+      <c r="T32" s="4" t="n"/>
+      <c r="U32" s="4" t="n"/>
+      <c r="V32" s="4" t="n"/>
+      <c r="W32" s="4" t="n"/>
+      <c r="X32" s="4" t="n"/>
+      <c r="Y32" s="4" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>0.0035275</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>0.9313</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>1.2291</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>0.4459</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>0.6656</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>0.8001</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>0.8594000000000001</v>
+      </c>
+      <c r="I33" s="5" t="n">
+        <v>0.777</v>
+      </c>
+      <c r="J33" s="5" t="n">
+        <v>0.7551</v>
+      </c>
+      <c r="K33" s="5" t="n">
+        <v>0.7659</v>
+      </c>
+      <c r="L33" s="5" t="n">
+        <v>0.7927999999999999</v>
+      </c>
+      <c r="M33" s="5" t="n">
+        <v>0.5609</v>
+      </c>
+      <c r="N33" s="5" t="n">
+        <v>0.9452</v>
+      </c>
+      <c r="O33" s="5" t="n">
+        <v>0.5503</v>
+      </c>
+      <c r="P33" s="5" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="Q33" s="5" t="n"/>
+      <c r="R33" s="5" t="n"/>
+      <c r="S33" s="5" t="n"/>
+      <c r="T33" s="5" t="n"/>
+      <c r="U33" s="5" t="n"/>
+      <c r="V33" s="5" t="n"/>
+      <c r="W33" s="5" t="n"/>
+      <c r="X33" s="5" t="n"/>
+      <c r="Y33" s="5" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="4" t="n">
+        <v>0.00348</v>
+      </c>
+      <c r="C34" s="4" t="n">
+        <v>1.0752</v>
+      </c>
+      <c r="D34" s="4" t="n">
+        <v>1.2274</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>0.6895</v>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>0.6642</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>0.8915999999999999</v>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>0.8593</v>
+      </c>
+      <c r="I34" s="4" t="n">
+        <v>0.7823</v>
+      </c>
+      <c r="J34" s="4" t="n">
+        <v>0.749</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>0.7653</v>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>0.7943</v>
+      </c>
+      <c r="M34" s="4" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="N34" s="4" t="n">
+        <v>0.9465</v>
+      </c>
+      <c r="O34" s="4" t="n">
+        <v>0.5518999999999999</v>
+      </c>
+      <c r="P34" s="4" t="n">
+        <v>0.9458</v>
+      </c>
+      <c r="Q34" s="4" t="n"/>
+      <c r="R34" s="4" t="n"/>
+      <c r="S34" s="4" t="n"/>
+      <c r="T34" s="4" t="n"/>
+      <c r="U34" s="4" t="n"/>
+      <c r="V34" s="4" t="n"/>
+      <c r="W34" s="4" t="n"/>
+      <c r="X34" s="4" t="n"/>
+      <c r="Y34" s="4" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>0.0034325</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>1.3043</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>1.2262</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>0.5705</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0.663</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>0.8679</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>0.8591</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>0.7187</v>
+      </c>
+      <c r="J35" s="5" t="n">
+        <v>0.7904</v>
+      </c>
+      <c r="K35" s="5" t="n">
+        <v>0.7528</v>
+      </c>
+      <c r="L35" s="5" t="n">
+        <v>0.7947</v>
+      </c>
+      <c r="M35" s="5" t="n">
+        <v>0.5628</v>
+      </c>
+      <c r="N35" s="5" t="n">
+        <v>0.947</v>
+      </c>
+      <c r="O35" s="5" t="n">
+        <v>0.5526</v>
+      </c>
+      <c r="P35" s="5" t="n">
+        <v>0.8806</v>
+      </c>
+      <c r="Q35" s="5" t="n"/>
+      <c r="R35" s="5" t="n"/>
+      <c r="S35" s="5" t="n"/>
+      <c r="T35" s="5" t="n"/>
+      <c r="U35" s="5" t="n"/>
+      <c r="V35" s="5" t="n"/>
+      <c r="W35" s="5" t="n"/>
+      <c r="X35" s="5" t="n"/>
+      <c r="Y35" s="5" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="4" t="n">
+        <v>0.003385</v>
+      </c>
+      <c r="C36" s="4" t="n">
+        <v>1.0279</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>1.2256</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>0.4795</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>0.6622</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>0.8339</v>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="I36" s="4" t="n">
+        <v>0.7185</v>
+      </c>
+      <c r="J36" s="4" t="n">
+        <v>0.7877999999999999</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>0.7514999999999999</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>0.7935</v>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>0.5618</v>
+      </c>
+      <c r="N36" s="4" t="n">
+        <v>0.9479</v>
+      </c>
+      <c r="O36" s="4" t="n">
+        <v>0.5532</v>
+      </c>
+      <c r="P36" s="4" t="n">
+        <v>0.8829</v>
+      </c>
+      <c r="Q36" s="4" t="n"/>
+      <c r="R36" s="4" t="n"/>
+      <c r="S36" s="4" t="n"/>
+      <c r="T36" s="4" t="n"/>
+      <c r="U36" s="4" t="n"/>
+      <c r="V36" s="4" t="n"/>
+      <c r="W36" s="4" t="n"/>
+      <c r="X36" s="4" t="n"/>
+      <c r="Y36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>0.0033375</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>1.1488</v>
+      </c>
+      <c r="D37" s="5" t="n">
+        <v>1.224</v>
+      </c>
+      <c r="E37" s="5" t="n">
+        <v>0.5137</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>0.6612</v>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>0.8148</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>0.8588</v>
+      </c>
+      <c r="I37" s="5" t="n">
+        <v>0.7289</v>
+      </c>
+      <c r="J37" s="5" t="n">
+        <v>0.7679</v>
+      </c>
+      <c r="K37" s="5" t="n">
+        <v>0.7479</v>
+      </c>
+      <c r="L37" s="5" t="n">
+        <v>0.7952</v>
+      </c>
+      <c r="M37" s="5" t="n">
+        <v>0.5619</v>
+      </c>
+      <c r="N37" s="5" t="n">
+        <v>0.9479</v>
+      </c>
+      <c r="O37" s="5" t="n">
+        <v>0.5538</v>
+      </c>
+      <c r="P37" s="5" t="n">
+        <v>0.9199000000000001</v>
+      </c>
+      <c r="Q37" s="5" t="n"/>
+      <c r="R37" s="5" t="n"/>
+      <c r="S37" s="5" t="n"/>
+      <c r="T37" s="5" t="n"/>
+      <c r="U37" s="5" t="n"/>
+      <c r="V37" s="5" t="n"/>
+      <c r="W37" s="5" t="n"/>
+      <c r="X37" s="5" t="n"/>
+      <c r="Y37" s="5" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="4" t="n">
+        <v>0.00329</v>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>1.2048</v>
+      </c>
+      <c r="D38" s="4" t="n">
+        <v>1.2224</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>0.5518</v>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>0.6598000000000001</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0.8178</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>0.8586</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>0.7309</v>
+      </c>
+      <c r="J38" s="4" t="n">
+        <v>0.7659</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>0.748</v>
+      </c>
+      <c r="L38" s="4" t="n">
+        <v>0.7946</v>
+      </c>
+      <c r="M38" s="4" t="n">
+        <v>0.5611</v>
+      </c>
+      <c r="N38" s="4" t="n">
+        <v>0.9482</v>
+      </c>
+      <c r="O38" s="4" t="n">
+        <v>0.5538999999999999</v>
+      </c>
+      <c r="P38" s="4" t="n">
+        <v>0.9243</v>
+      </c>
+      <c r="Q38" s="4" t="n"/>
+      <c r="R38" s="4" t="n"/>
+      <c r="S38" s="4" t="n"/>
+      <c r="T38" s="4" t="n"/>
+      <c r="U38" s="4" t="n"/>
+      <c r="V38" s="4" t="n"/>
+      <c r="W38" s="4" t="n"/>
+      <c r="X38" s="4" t="n"/>
+      <c r="Y38" s="4" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>0.0032425</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>1.3551</v>
+      </c>
+      <c r="D39" s="5" t="n">
+        <v>1.2219</v>
+      </c>
+      <c r="E39" s="5" t="n">
+        <v>0.6133999999999999</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>0.6597</v>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>0.853</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>0.8584000000000001</v>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>0.819</v>
+      </c>
+      <c r="J39" s="5" t="n">
+        <v>0.7016</v>
+      </c>
+      <c r="K39" s="5" t="n">
+        <v>0.7558</v>
+      </c>
+      <c r="L39" s="5" t="n">
+        <v>0.7964</v>
+      </c>
+      <c r="M39" s="5" t="n">
+        <v>0.5626</v>
+      </c>
+      <c r="N39" s="5" t="n">
+        <v>0.9483</v>
+      </c>
+      <c r="O39" s="5" t="n">
+        <v>0.5545</v>
+      </c>
+      <c r="P39" s="5" t="n">
+        <v>0.9664</v>
+      </c>
+      <c r="Q39" s="5" t="n"/>
+      <c r="R39" s="5" t="n"/>
+      <c r="S39" s="5" t="n"/>
+      <c r="T39" s="5" t="n"/>
+      <c r="U39" s="5" t="n"/>
+      <c r="V39" s="5" t="n"/>
+      <c r="W39" s="5" t="n"/>
+      <c r="X39" s="5" t="n"/>
+      <c r="Y39" s="5" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>0.003195</v>
+      </c>
+      <c r="C40" s="4" t="n">
+        <v>1.3031</v>
+      </c>
+      <c r="D40" s="4" t="n">
+        <v>1.2209</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>0.6873</v>
+      </c>
+      <c r="F40" s="4" t="n">
+        <v>0.6583</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>0.8468</v>
+      </c>
+      <c r="H40" s="4" t="n">
+        <v>0.8583</v>
+      </c>
+      <c r="I40" s="4" t="n">
+        <v>0.8168</v>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>0.7028</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>0.7556</v>
+      </c>
+      <c r="L40" s="4" t="n">
+        <v>0.796</v>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>0.5634</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>0.9484</v>
+      </c>
+      <c r="O40" s="4" t="n">
+        <v>0.5548</v>
+      </c>
+      <c r="P40" s="4" t="n">
+        <v>0.9661999999999999</v>
+      </c>
+      <c r="Q40" s="4" t="n"/>
+      <c r="R40" s="4" t="n"/>
+      <c r="S40" s="4" t="n"/>
+      <c r="T40" s="4" t="n"/>
+      <c r="U40" s="4" t="n"/>
+      <c r="V40" s="4" t="n"/>
+      <c r="W40" s="4" t="n"/>
+      <c r="X40" s="4" t="n"/>
+      <c r="Y40" s="4" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>0.0031475</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>1.1516</v>
+      </c>
+      <c r="D41" s="5" t="n">
+        <v>1.2199</v>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>0.5188</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>0.6572</v>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>0.8491</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>0.8581</v>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>0.8166</v>
+      </c>
+      <c r="J41" s="5" t="n">
+        <v>0.7028</v>
+      </c>
+      <c r="K41" s="5" t="n">
+        <v>0.7554</v>
+      </c>
+      <c r="L41" s="5" t="n">
+        <v>0.7946</v>
+      </c>
+      <c r="M41" s="5" t="n">
+        <v>0.5624</v>
+      </c>
+      <c r="N41" s="5" t="n">
+        <v>0.9487</v>
+      </c>
+      <c r="O41" s="5" t="n">
+        <v>0.5546</v>
+      </c>
+      <c r="P41" s="5" t="n">
+        <v>0.9663</v>
+      </c>
+      <c r="Q41" s="5" t="n"/>
+      <c r="R41" s="5" t="n"/>
+      <c r="S41" s="5" t="n"/>
+      <c r="T41" s="5" t="n"/>
+      <c r="U41" s="5" t="n"/>
+      <c r="V41" s="5" t="n"/>
+      <c r="W41" s="5" t="n"/>
+      <c r="X41" s="5" t="n"/>
+      <c r="Y41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="4" t="n">
+        <v>0.0031</v>
+      </c>
+      <c r="C42" s="4" t="n">
+        <v>1.0409</v>
+      </c>
+      <c r="D42" s="4" t="n">
+        <v>1.2182</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>0.4947</v>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>0.6561</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>0.8714</v>
+      </c>
+      <c r="H42" s="4" t="n">
+        <v>0.8579</v>
+      </c>
+      <c r="I42" s="4" t="n">
+        <v>0.8155</v>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>0.7028</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>0.755</v>
+      </c>
+      <c r="L42" s="4" t="n">
+        <v>0.7945</v>
+      </c>
+      <c r="M42" s="4" t="n">
+        <v>0.5624</v>
+      </c>
+      <c r="N42" s="4" t="n">
+        <v>0.9484</v>
+      </c>
+      <c r="O42" s="4" t="n">
+        <v>0.5546</v>
+      </c>
+      <c r="P42" s="4" t="n">
+        <v>0.9661</v>
+      </c>
+      <c r="Q42" s="4" t="n"/>
+      <c r="R42" s="4" t="n"/>
+      <c r="S42" s="4" t="n"/>
+      <c r="T42" s="4" t="n"/>
+      <c r="U42" s="4" t="n"/>
+      <c r="V42" s="4" t="n"/>
+      <c r="W42" s="4" t="n"/>
+      <c r="X42" s="4" t="n"/>
+      <c r="Y42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>0.0030525</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>1.0969</v>
+      </c>
+      <c r="D43" s="5" t="n">
+        <v>1.217</v>
+      </c>
+      <c r="E43" s="5" t="n">
+        <v>0.5278</v>
+      </c>
+      <c r="F43" s="5" t="n">
+        <v>0.6549</v>
+      </c>
+      <c r="G43" s="5" t="n">
+        <v>0.858</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>0.8577</v>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>0.7367</v>
+      </c>
+      <c r="J43" s="5" t="n">
+        <v>0.7663</v>
+      </c>
+      <c r="K43" s="5" t="n">
+        <v>0.7512</v>
+      </c>
+      <c r="L43" s="5" t="n">
+        <v>0.7947</v>
+      </c>
+      <c r="M43" s="5" t="n">
+        <v>0.5623</v>
+      </c>
+      <c r="N43" s="5" t="n">
+        <v>0.9484</v>
+      </c>
+      <c r="O43" s="5" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="P43" s="5" t="n">
+        <v>0.9179</v>
+      </c>
+      <c r="Q43" s="5" t="n"/>
+      <c r="R43" s="5" t="n"/>
+      <c r="S43" s="5" t="n"/>
+      <c r="T43" s="5" t="n"/>
+      <c r="U43" s="5" t="n"/>
+      <c r="V43" s="5" t="n"/>
+      <c r="W43" s="5" t="n"/>
+      <c r="X43" s="5" t="n"/>
+      <c r="Y43" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="4" t="n">
+        <v>0.003005</v>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>1.3017</v>
+      </c>
+      <c r="D44" s="4" t="n">
+        <v>1.2166</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>0.5416</v>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>0.6534</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>0.8907</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>0.8576</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>0.7147</v>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>0.773</v>
+      </c>
+      <c r="K44" s="4" t="n">
+        <v>0.7427</v>
+      </c>
+      <c r="L44" s="4" t="n">
+        <v>0.7937</v>
+      </c>
+      <c r="M44" s="4" t="n">
+        <v>0.5606</v>
+      </c>
+      <c r="N44" s="4" t="n">
+        <v>0.9484</v>
+      </c>
+      <c r="O44" s="4" t="n">
+        <v>0.5557</v>
+      </c>
+      <c r="P44" s="4" t="n">
+        <v>0.9009</v>
+      </c>
+      <c r="Q44" s="4" t="n"/>
+      <c r="R44" s="4" t="n"/>
+      <c r="S44" s="4" t="n"/>
+      <c r="T44" s="4" t="n"/>
+      <c r="U44" s="4" t="n"/>
+      <c r="V44" s="4" t="n"/>
+      <c r="W44" s="4" t="n"/>
+      <c r="X44" s="4" t="n"/>
+      <c r="Y44" s="4" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>0.0029575</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>1.3426</v>
+      </c>
+      <c r="D45" s="5" t="n">
+        <v>1.2156</v>
+      </c>
+      <c r="E45" s="5" t="n">
+        <v>0.6175</v>
+      </c>
+      <c r="F45" s="5" t="n">
+        <v>0.6529</v>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>0.8949</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>0.8576</v>
+      </c>
+      <c r="I45" s="5" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="J45" s="5" t="n">
+        <v>0.7904</v>
+      </c>
+      <c r="K45" s="5" t="n">
+        <v>0.7492</v>
+      </c>
+      <c r="L45" s="5" t="n">
+        <v>0.7929</v>
+      </c>
+      <c r="M45" s="5" t="n">
+        <v>0.5595</v>
+      </c>
+      <c r="N45" s="5" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="O45" s="5" t="n">
+        <v>0.5561</v>
+      </c>
+      <c r="P45" s="5" t="n">
+        <v>0.8857</v>
+      </c>
+      <c r="Q45" s="5" t="n"/>
+      <c r="R45" s="5" t="n"/>
+      <c r="S45" s="5" t="n"/>
+      <c r="T45" s="5" t="n"/>
+      <c r="U45" s="5" t="n"/>
+      <c r="V45" s="5" t="n"/>
+      <c r="W45" s="5" t="n"/>
+      <c r="X45" s="5" t="n"/>
+      <c r="Y45" s="5" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="4" t="n">
+        <v>0.00291</v>
+      </c>
+      <c r="C46" s="4" t="n">
+        <v>0.9975000000000001</v>
+      </c>
+      <c r="D46" s="4" t="n">
+        <v>1.215</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>0.4506</v>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>0.6526</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>0.8002</v>
+      </c>
+      <c r="H46" s="4" t="n">
+        <v>0.8574000000000001</v>
+      </c>
+      <c r="I46" s="4" t="n">
+        <v>0.7030999999999999</v>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>0.7914</v>
+      </c>
+      <c r="K46" s="4" t="n">
+        <v>0.7446</v>
+      </c>
+      <c r="L46" s="4" t="n">
+        <v>0.7915</v>
+      </c>
+      <c r="M46" s="4" t="n">
+        <v>0.5587</v>
+      </c>
+      <c r="N46" s="4" t="n">
+        <v>0.949</v>
+      </c>
+      <c r="O46" s="4" t="n">
+        <v>0.5561</v>
+      </c>
+      <c r="P46" s="4" t="n">
+        <v>0.8813</v>
+      </c>
+      <c r="Q46" s="4" t="n"/>
+      <c r="R46" s="4" t="n"/>
+      <c r="S46" s="4" t="n"/>
+      <c r="T46" s="4" t="n"/>
+      <c r="U46" s="4" t="n"/>
+      <c r="V46" s="4" t="n"/>
+      <c r="W46" s="4" t="n"/>
+      <c r="X46" s="4" t="n"/>
+      <c r="Y46" s="4" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>0.00291</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>0.9975000000000001</v>
+      </c>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n">
+        <v>0.4506</v>
+      </c>
+      <c r="F47" s="5" t="n"/>
+      <c r="G47" s="5" t="n">
+        <v>0.8002</v>
+      </c>
+      <c r="H47" s="5" t="n"/>
+      <c r="I47" s="5" t="n">
+        <v>0.8265</v>
+      </c>
+      <c r="J47" s="5" t="n">
+        <v>0.8001</v>
+      </c>
+      <c r="K47" s="5" t="n">
+        <v>0.8131</v>
+      </c>
+      <c r="L47" s="5" t="n">
+        <v>0.8201000000000001</v>
+      </c>
+      <c r="M47" s="5" t="n">
+        <v>0.5712</v>
+      </c>
+      <c r="N47" s="5" t="n">
+        <v>0.9374</v>
+      </c>
+      <c r="O47" s="5" t="n">
+        <v>0.5315</v>
+      </c>
+      <c r="P47" s="5" t="n">
+        <v>0.9292</v>
+      </c>
+      <c r="Q47" s="5" t="n"/>
+      <c r="R47" s="5" t="n"/>
+      <c r="S47" s="5" t="n"/>
+      <c r="T47" s="5" t="n"/>
+      <c r="U47" s="5" t="n"/>
+      <c r="V47" s="5" t="n"/>
+      <c r="W47" s="5" t="n"/>
+      <c r="X47" s="5" t="n"/>
+      <c r="Y47" s="5" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>